<commit_message>
Generate report Thanh toan Khoa Luan
</commit_message>
<xml_diff>
--- a/static/samples/Data_RaDeDuyetDeChamThi.xlsx
+++ b/static/samples/Data_RaDeDuyetDeChamThi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\hienlth.io.vn\FIT_Tools\tools\static\samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39C2E93B-ABB9-4A3A-B670-E21C5EE19F3B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{050536B2-EBD4-4DBB-9CEB-896E889716BA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,55 +24,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author/>
-  </authors>
-  <commentList>
-    <comment ref="E2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>======
-ID#AAAB3yRVNx8
-Lương Trần Hy Hiến - Khoa CNTT    (2026-04-20 15:31:21)
-không có trong QC CTNB 2025</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>======
-ID#AAAB3yRVNyA
-Lương Trần Hy Hiến - Khoa CNTT    (2026-04-20 15:31:27)
-không có trong QC CTNB 2025</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-  <extLst>
-    <ext xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mhJdSry2SWv+B7k8ICBMyXz1kUagA=="/>
-    </ext>
-  </extLst>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Ra đề tự luận</t>
   </si>
@@ -111,6 +64,15 @@
   </si>
   <si>
     <t>X</t>
+  </si>
+  <si>
+    <t>Năm học</t>
+  </si>
+  <si>
+    <t>2025 - 2026</t>
+  </si>
+  <si>
+    <t>Học kỳ</t>
   </si>
 </sst>
 </file>
@@ -193,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -222,6 +184,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -436,7 +402,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -456,8 +422,18 @@
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="C1" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="2" spans="1:8" ht="14.1" x14ac:dyDescent="0.5">
       <c r="A2" s="4" t="s">
@@ -5387,6 +5363,5 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update in sao de, coi thi
</commit_message>
<xml_diff>
--- a/static/samples/Data_RaDeDuyetDeChamThi.xlsx
+++ b/static/samples/Data_RaDeDuyetDeChamThi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\hienlth.io.vn\FIT_Tools\tools\static\samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{050536B2-EBD4-4DBB-9CEB-896E889716BA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D572B25-CAAE-49F9-B3D7-9A4502211676}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Ra đề tự luận</t>
   </si>
@@ -73,6 +73,15 @@
   </si>
   <si>
     <t>Học kỳ</t>
+  </si>
+  <si>
+    <t>In sao đề</t>
+  </si>
+  <si>
+    <t>Coi thi trên 90 phút</t>
+  </si>
+  <si>
+    <t>Coi thi đến 90 phút</t>
   </si>
 </sst>
 </file>
@@ -406,7 +415,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:H972"/>
+  <dimension ref="A1:K972"/>
   <sheetFormatPr defaultColWidth="14.41796875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9" style="3" customWidth="1"/>
@@ -415,10 +424,13 @@
     <col min="4" max="6" width="14.41796875" style="2"/>
     <col min="7" max="7" width="16.41796875" style="2" customWidth="1"/>
     <col min="8" max="8" width="17.68359375" style="2" customWidth="1"/>
-    <col min="9" max="16384" width="14.41796875" style="2"/>
+    <col min="9" max="9" width="9.26171875" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.5234375" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.68359375" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="14.41796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -435,7 +447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="14.1" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:11" ht="14.1" x14ac:dyDescent="0.5">
       <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
@@ -460,8 +472,17 @@
       <c r="H2" s="4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="13.8" x14ac:dyDescent="0.45">
+      <c r="I2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="13.8" x14ac:dyDescent="0.45">
       <c r="A3" s="6">
         <v>1506</v>
       </c>
@@ -478,8 +499,11 @@
       </c>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
-    </row>
-    <row r="4" spans="1:8" ht="13.8" x14ac:dyDescent="0.45">
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+    </row>
+    <row r="4" spans="1:11" ht="13.8" x14ac:dyDescent="0.45">
       <c r="A4" s="6">
         <v>1642</v>
       </c>
@@ -496,8 +520,11 @@
       </c>
       <c r="G4" s="9"/>
       <c r="H4" s="10"/>
-    </row>
-    <row r="5" spans="1:8" ht="13.8" x14ac:dyDescent="0.45">
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+    </row>
+    <row r="5" spans="1:11" ht="13.8" x14ac:dyDescent="0.45">
       <c r="A5" s="6">
         <v>9777</v>
       </c>
@@ -516,8 +543,11 @@
       </c>
       <c r="G5" s="9"/>
       <c r="H5" s="10"/>
-    </row>
-    <row r="6" spans="1:8" ht="14.1" x14ac:dyDescent="0.5">
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+    </row>
+    <row r="6" spans="1:11" ht="14.1" x14ac:dyDescent="0.5">
       <c r="B6" s="11"/>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -526,7 +556,7 @@
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B7" s="11"/>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -535,47 +565,47 @@
       <c r="G7" s="11"/>
       <c r="H7" s="11"/>
     </row>
-    <row r="8" spans="1:8" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="13.8" x14ac:dyDescent="0.45">
       <c r="D8" s="12"/>
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
     </row>
-    <row r="9" spans="1:8" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="13.8" x14ac:dyDescent="0.45">
       <c r="D9" s="12"/>
       <c r="E9" s="12"/>
       <c r="F9" s="12"/>
     </row>
-    <row r="10" spans="1:8" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="13.8" x14ac:dyDescent="0.45">
       <c r="D10" s="12"/>
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
     </row>
-    <row r="11" spans="1:8" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="13.8" x14ac:dyDescent="0.45">
       <c r="D11" s="12"/>
       <c r="E11" s="12"/>
       <c r="F11" s="12"/>
     </row>
-    <row r="12" spans="1:8" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="13.8" x14ac:dyDescent="0.45">
       <c r="D12" s="12"/>
       <c r="E12" s="12"/>
       <c r="F12" s="12"/>
     </row>
-    <row r="13" spans="1:8" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="13.8" x14ac:dyDescent="0.45">
       <c r="D13" s="12"/>
       <c r="E13" s="12"/>
       <c r="F13" s="12"/>
     </row>
-    <row r="14" spans="1:8" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="13.8" x14ac:dyDescent="0.45">
       <c r="D14" s="12"/>
       <c r="E14" s="12"/>
       <c r="F14" s="12"/>
     </row>
-    <row r="15" spans="1:8" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="13.8" x14ac:dyDescent="0.45">
       <c r="D15" s="12"/>
       <c r="E15" s="12"/>
       <c r="F15" s="12"/>
     </row>
-    <row r="16" spans="1:8" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="13.8" x14ac:dyDescent="0.45">
       <c r="D16" s="12"/>
       <c r="E16" s="12"/>
       <c r="F16" s="12"/>

</xml_diff>